<commit_message>
Commit At 2026-09-23 15:46:11
</commit_message>
<xml_diff>
--- a/数据/无人机应急物资运输基础数据/物资需求与配送时限.xlsx
+++ b/数据/无人机应急物资运输基础数据/物资需求与配送时限.xlsx
@@ -1,13 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SF_Dir\第二十三届中国研究生数学建模竞赛 - 中文题目\中文题目\D题\HUAWEI-CUP\数据\无人机应急物资运输基础数据\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="15300"/>
+    <workbookView windowWidth="25600" windowHeight="12080"/>
   </bookViews>
   <sheets>
-    <sheet name="数据" sheetId="1" r:id="rId1"/>
+    <sheet name="各服务区物资需求" sheetId="1" r:id="rId1"/>
     <sheet name="逐箱货箱清单" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -784,12 +789,18 @@
       <charset val="134"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1110,7 +1121,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1134,16 +1145,16 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1152,90 +1163,90 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1262,7 +1273,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="49" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="49" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1285,6 +1296,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="6" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1759,17 +1788,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I54"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="12" style="10" customWidth="1"/>
-    <col min="2" max="2" width="16" style="10" customWidth="1"/>
-    <col min="3" max="3" width="12" style="10" customWidth="1"/>
-    <col min="4" max="4" width="16" style="10" customWidth="1"/>
-    <col min="5" max="6" width="15.9" style="10" customWidth="1"/>
-    <col min="7" max="7" width="14" style="10" customWidth="1"/>
-    <col min="8" max="8" width="17" style="10" customWidth="1"/>
-    <col min="9" max="9" width="17" style="9" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="10"/>
+    <col min="1" max="1" width="12" style="9" customWidth="1"/>
+    <col min="2" max="2" width="16" style="9" customWidth="1"/>
+    <col min="3" max="3" width="12" style="9" customWidth="1"/>
+    <col min="4" max="4" width="16" style="9" customWidth="1"/>
+    <col min="5" max="6" width="15.9" style="9" customWidth="1"/>
+    <col min="7" max="7" width="14" style="9" customWidth="1"/>
+    <col min="8" max="9" width="17" style="9" customWidth="1"/>
+    <col min="10" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
     <row r="1" s="9" customFormat="1" ht="32" customHeight="1" spans="1:9">
@@ -1913,115 +1941,115 @@
         <v>10800</v>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1" spans="1:9">
-      <c r="A6" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="13" t="s">
+    <row r="6" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A6" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="14">
-        <v>1</v>
-      </c>
-      <c r="D6" s="14">
-        <v>1</v>
-      </c>
-      <c r="E6" s="15">
+      <c r="C6" s="20">
+        <v>1</v>
+      </c>
+      <c r="D6" s="20">
+        <v>1</v>
+      </c>
+      <c r="E6" s="21">
         <v>3</v>
       </c>
-      <c r="F6" s="16">
+      <c r="F6" s="22">
         <v>0.012</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="20">
         <v>24</v>
       </c>
-      <c r="H6" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I6" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:9">
-      <c r="A7" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="13" t="s">
+      <c r="H6" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I6" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="7" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A7" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="20">
         <v>4</v>
       </c>
-      <c r="D7" s="14">
-        <v>1</v>
-      </c>
-      <c r="E7" s="15">
-        <v>14</v>
-      </c>
-      <c r="F7" s="16">
+      <c r="D7" s="20">
+        <v>1</v>
+      </c>
+      <c r="E7" s="21">
+        <v>14</v>
+      </c>
+      <c r="F7" s="22">
         <v>0.027</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="20">
         <v>12</v>
       </c>
-      <c r="H7" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I7" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:9">
-      <c r="A8" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="13" t="s">
+      <c r="H7" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I7" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="8" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A8" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="20">
         <v>2</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="20">
         <v>0</v>
       </c>
-      <c r="E8" s="15">
-        <v>8</v>
-      </c>
-      <c r="F8" s="16">
+      <c r="E8" s="21">
+        <v>8</v>
+      </c>
+      <c r="F8" s="22">
         <v>0.028</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="20">
         <v>10</v>
       </c>
-      <c r="H8" s="17"/>
-      <c r="I8" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:9">
-      <c r="A9" s="13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="13" t="s">
+      <c r="H8" s="23"/>
+      <c r="I8" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="9" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A9" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="14">
-        <v>1</v>
-      </c>
-      <c r="D9" s="14">
+      <c r="C9" s="20">
+        <v>1</v>
+      </c>
+      <c r="D9" s="20">
         <v>0</v>
       </c>
-      <c r="E9" s="15">
+      <c r="E9" s="21">
         <v>6</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="22">
         <v>0.035</v>
       </c>
-      <c r="G9" s="14">
-        <v>8</v>
-      </c>
-      <c r="H9" s="17"/>
-      <c r="I9" s="18">
+      <c r="G9" s="20">
+        <v>8</v>
+      </c>
+      <c r="H9" s="23"/>
+      <c r="I9" s="24">
         <v>10800</v>
       </c>
     </row>
@@ -2137,115 +2165,115 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1" spans="1:9">
-      <c r="A14" s="13" t="s">
+    <row r="14" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A14" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C14" s="14">
-        <v>1</v>
-      </c>
-      <c r="D14" s="14">
-        <v>1</v>
-      </c>
-      <c r="E14" s="15">
+      <c r="C14" s="20">
+        <v>1</v>
+      </c>
+      <c r="D14" s="20">
+        <v>1</v>
+      </c>
+      <c r="E14" s="21">
         <v>3</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="22">
         <v>0.012</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="20">
         <v>20</v>
       </c>
-      <c r="H14" s="17">
-        <v>7200</v>
-      </c>
-      <c r="I14" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:9">
-      <c r="A15" s="13" t="s">
+      <c r="H14" s="23">
+        <v>7200</v>
+      </c>
+      <c r="I14" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="15" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A15" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="20">
         <v>3</v>
       </c>
-      <c r="D15" s="14">
-        <v>1</v>
-      </c>
-      <c r="E15" s="15">
-        <v>14</v>
-      </c>
-      <c r="F15" s="16">
+      <c r="D15" s="20">
+        <v>1</v>
+      </c>
+      <c r="E15" s="21">
+        <v>14</v>
+      </c>
+      <c r="F15" s="22">
         <v>0.027</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="20">
         <v>10</v>
       </c>
-      <c r="H15" s="17">
-        <v>7200</v>
-      </c>
-      <c r="I15" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1" spans="1:9">
-      <c r="A16" s="13" t="s">
+      <c r="H15" s="23">
+        <v>7200</v>
+      </c>
+      <c r="I15" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="16" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A16" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="14">
-        <v>1</v>
-      </c>
-      <c r="D16" s="14">
+      <c r="C16" s="20">
+        <v>1</v>
+      </c>
+      <c r="D16" s="20">
         <v>0</v>
       </c>
-      <c r="E16" s="15">
-        <v>8</v>
-      </c>
-      <c r="F16" s="16">
+      <c r="E16" s="21">
+        <v>8</v>
+      </c>
+      <c r="F16" s="22">
         <v>0.028</v>
       </c>
-      <c r="G16" s="14">
-        <v>8</v>
-      </c>
-      <c r="H16" s="17"/>
-      <c r="I16" s="18">
+      <c r="G16" s="20">
+        <v>8</v>
+      </c>
+      <c r="H16" s="23"/>
+      <c r="I16" s="24">
         <v>10800</v>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1" spans="1:9">
-      <c r="A17" s="13" t="s">
+    <row r="17" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A17" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="14">
-        <v>1</v>
-      </c>
-      <c r="D17" s="14">
+      <c r="C17" s="20">
+        <v>1</v>
+      </c>
+      <c r="D17" s="20">
         <v>0</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="21">
         <v>6</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="22">
         <v>0.035</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="20">
         <v>6</v>
       </c>
-      <c r="H17" s="17"/>
-      <c r="I17" s="18">
+      <c r="H17" s="23"/>
+      <c r="I17" s="24">
         <v>14400</v>
       </c>
     </row>
@@ -2361,115 +2389,115 @@
         <v>18000</v>
       </c>
     </row>
-    <row r="22" ht="22" customHeight="1" spans="1:9">
-      <c r="A22" s="13" t="s">
+    <row r="22" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A22" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C22" s="14">
-        <v>1</v>
-      </c>
-      <c r="D22" s="14">
-        <v>1</v>
-      </c>
-      <c r="E22" s="15">
+      <c r="C22" s="20">
+        <v>1</v>
+      </c>
+      <c r="D22" s="20">
+        <v>1</v>
+      </c>
+      <c r="E22" s="21">
         <v>3</v>
       </c>
-      <c r="F22" s="16">
+      <c r="F22" s="22">
         <v>0.012</v>
       </c>
-      <c r="G22" s="14">
+      <c r="G22" s="20">
         <v>24</v>
       </c>
-      <c r="H22" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I22" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1" spans="1:9">
-      <c r="A23" s="13" t="s">
+      <c r="H22" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I22" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="23" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A23" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B23" s="13" t="s">
+      <c r="B23" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="20">
         <v>3</v>
       </c>
-      <c r="D23" s="14">
-        <v>1</v>
-      </c>
-      <c r="E23" s="15">
-        <v>14</v>
-      </c>
-      <c r="F23" s="16">
+      <c r="D23" s="20">
+        <v>1</v>
+      </c>
+      <c r="E23" s="21">
+        <v>14</v>
+      </c>
+      <c r="F23" s="22">
         <v>0.027</v>
       </c>
-      <c r="G23" s="14">
+      <c r="G23" s="20">
         <v>12</v>
       </c>
-      <c r="H23" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I23" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="24" ht="22" customHeight="1" spans="1:9">
-      <c r="A24" s="13" t="s">
+      <c r="H23" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I23" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="24" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A24" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C24" s="14">
-        <v>1</v>
-      </c>
-      <c r="D24" s="14">
+      <c r="C24" s="20">
+        <v>1</v>
+      </c>
+      <c r="D24" s="20">
         <v>0</v>
       </c>
-      <c r="E24" s="15">
-        <v>8</v>
-      </c>
-      <c r="F24" s="16">
+      <c r="E24" s="21">
+        <v>8</v>
+      </c>
+      <c r="F24" s="22">
         <v>0.028</v>
       </c>
-      <c r="G24" s="14">
+      <c r="G24" s="20">
         <v>10</v>
       </c>
-      <c r="H24" s="17"/>
-      <c r="I24" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="25" ht="22" customHeight="1" spans="1:9">
-      <c r="A25" s="13" t="s">
+      <c r="H24" s="23"/>
+      <c r="I24" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="25" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A25" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="13" t="s">
+      <c r="B25" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C25" s="14">
-        <v>1</v>
-      </c>
-      <c r="D25" s="14">
+      <c r="C25" s="20">
+        <v>1</v>
+      </c>
+      <c r="D25" s="20">
         <v>0</v>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="21">
         <v>6</v>
       </c>
-      <c r="F25" s="16">
+      <c r="F25" s="22">
         <v>0.035</v>
       </c>
-      <c r="G25" s="14">
-        <v>8</v>
-      </c>
-      <c r="H25" s="17"/>
-      <c r="I25" s="18">
+      <c r="G25" s="20">
+        <v>8</v>
+      </c>
+      <c r="H25" s="23"/>
+      <c r="I25" s="24">
         <v>10800</v>
       </c>
     </row>
@@ -2585,115 +2613,115 @@
         <v>10800</v>
       </c>
     </row>
-    <row r="30" ht="22" customHeight="1" spans="1:9">
-      <c r="A30" s="13" t="s">
+    <row r="30" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A30" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="14">
-        <v>1</v>
-      </c>
-      <c r="D30" s="14">
-        <v>1</v>
-      </c>
-      <c r="E30" s="15">
+      <c r="C30" s="20">
+        <v>1</v>
+      </c>
+      <c r="D30" s="20">
+        <v>1</v>
+      </c>
+      <c r="E30" s="21">
         <v>3</v>
       </c>
-      <c r="F30" s="16">
+      <c r="F30" s="22">
         <v>0.012</v>
       </c>
-      <c r="G30" s="14">
+      <c r="G30" s="20">
         <v>20</v>
       </c>
-      <c r="H30" s="17">
-        <v>7200</v>
-      </c>
-      <c r="I30" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1" spans="1:9">
-      <c r="A31" s="13" t="s">
+      <c r="H30" s="23">
+        <v>7200</v>
+      </c>
+      <c r="I30" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="31" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A31" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="20">
         <v>2</v>
       </c>
-      <c r="D31" s="14">
-        <v>1</v>
-      </c>
-      <c r="E31" s="15">
-        <v>14</v>
-      </c>
-      <c r="F31" s="16">
+      <c r="D31" s="20">
+        <v>1</v>
+      </c>
+      <c r="E31" s="21">
+        <v>14</v>
+      </c>
+      <c r="F31" s="22">
         <v>0.027</v>
       </c>
-      <c r="G31" s="14">
+      <c r="G31" s="20">
         <v>10</v>
       </c>
-      <c r="H31" s="17">
-        <v>7200</v>
-      </c>
-      <c r="I31" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="32" ht="22" customHeight="1" spans="1:9">
-      <c r="A32" s="13" t="s">
+      <c r="H31" s="23">
+        <v>7200</v>
+      </c>
+      <c r="I31" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="32" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A32" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C32" s="14">
-        <v>1</v>
-      </c>
-      <c r="D32" s="14">
+      <c r="C32" s="20">
+        <v>1</v>
+      </c>
+      <c r="D32" s="20">
         <v>0</v>
       </c>
-      <c r="E32" s="15">
-        <v>8</v>
-      </c>
-      <c r="F32" s="16">
+      <c r="E32" s="21">
+        <v>8</v>
+      </c>
+      <c r="F32" s="22">
         <v>0.028</v>
       </c>
-      <c r="G32" s="14">
-        <v>8</v>
-      </c>
-      <c r="H32" s="17"/>
-      <c r="I32" s="18">
+      <c r="G32" s="20">
+        <v>8</v>
+      </c>
+      <c r="H32" s="23"/>
+      <c r="I32" s="24">
         <v>10800</v>
       </c>
     </row>
-    <row r="33" ht="22" customHeight="1" spans="1:9">
-      <c r="A33" s="13" t="s">
+    <row r="33" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A33" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C33" s="14">
-        <v>1</v>
-      </c>
-      <c r="D33" s="14">
+      <c r="C33" s="20">
+        <v>1</v>
+      </c>
+      <c r="D33" s="20">
         <v>0</v>
       </c>
-      <c r="E33" s="15">
+      <c r="E33" s="21">
         <v>6</v>
       </c>
-      <c r="F33" s="16">
+      <c r="F33" s="22">
         <v>0.035</v>
       </c>
-      <c r="G33" s="14">
+      <c r="G33" s="20">
         <v>6</v>
       </c>
-      <c r="H33" s="17"/>
-      <c r="I33" s="18">
+      <c r="H33" s="23"/>
+      <c r="I33" s="24">
         <v>14400</v>
       </c>
     </row>
@@ -2782,88 +2810,88 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="37" ht="22" customHeight="1" spans="1:9">
-      <c r="A37" s="13" t="s">
+    <row r="37" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A37" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B37" s="13" t="s">
+      <c r="B37" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C37" s="14">
-        <v>1</v>
-      </c>
-      <c r="D37" s="14">
-        <v>1</v>
-      </c>
-      <c r="E37" s="15">
+      <c r="C37" s="20">
+        <v>1</v>
+      </c>
+      <c r="D37" s="20">
+        <v>1</v>
+      </c>
+      <c r="E37" s="21">
         <v>3</v>
       </c>
-      <c r="F37" s="16">
+      <c r="F37" s="22">
         <v>0.012</v>
       </c>
-      <c r="G37" s="14">
+      <c r="G37" s="20">
         <v>24</v>
       </c>
-      <c r="H37" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I37" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="38" ht="22" customHeight="1" spans="1:9">
-      <c r="A38" s="13" t="s">
+      <c r="H37" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I37" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="38" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A38" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B38" s="13" t="s">
+      <c r="B38" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C38" s="14">
-        <v>1</v>
-      </c>
-      <c r="D38" s="14">
-        <v>1</v>
-      </c>
-      <c r="E38" s="15">
-        <v>14</v>
-      </c>
-      <c r="F38" s="16">
+      <c r="C38" s="20">
+        <v>1</v>
+      </c>
+      <c r="D38" s="20">
+        <v>1</v>
+      </c>
+      <c r="E38" s="21">
+        <v>14</v>
+      </c>
+      <c r="F38" s="22">
         <v>0.027</v>
       </c>
-      <c r="G38" s="14">
+      <c r="G38" s="20">
         <v>12</v>
       </c>
-      <c r="H38" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I38" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="39" ht="22" customHeight="1" spans="1:9">
-      <c r="A39" s="13" t="s">
+      <c r="H38" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I38" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="39" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A39" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="B39" s="13" t="s">
+      <c r="B39" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C39" s="14">
-        <v>1</v>
-      </c>
-      <c r="D39" s="14">
+      <c r="C39" s="20">
+        <v>1</v>
+      </c>
+      <c r="D39" s="20">
         <v>0</v>
       </c>
-      <c r="E39" s="15">
-        <v>8</v>
-      </c>
-      <c r="F39" s="16">
+      <c r="E39" s="21">
+        <v>8</v>
+      </c>
+      <c r="F39" s="22">
         <v>0.028</v>
       </c>
-      <c r="G39" s="14">
+      <c r="G39" s="20">
         <v>10</v>
       </c>
-      <c r="H39" s="17"/>
-      <c r="I39" s="18">
+      <c r="H39" s="23"/>
+      <c r="I39" s="24">
         <v>7200</v>
       </c>
     </row>
@@ -2952,88 +2980,88 @@
         <v>14400</v>
       </c>
     </row>
-    <row r="43" ht="22" customHeight="1" spans="1:9">
-      <c r="A43" s="13" t="s">
+    <row r="43" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A43" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B43" s="13" t="s">
+      <c r="B43" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C43" s="14">
-        <v>1</v>
-      </c>
-      <c r="D43" s="14">
-        <v>1</v>
-      </c>
-      <c r="E43" s="15">
+      <c r="C43" s="20">
+        <v>1</v>
+      </c>
+      <c r="D43" s="20">
+        <v>1</v>
+      </c>
+      <c r="E43" s="21">
         <v>3</v>
       </c>
-      <c r="F43" s="16">
+      <c r="F43" s="22">
         <v>0.012</v>
       </c>
-      <c r="G43" s="14">
+      <c r="G43" s="20">
         <v>22</v>
       </c>
-      <c r="H43" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I43" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="44" ht="22" customHeight="1" spans="1:9">
-      <c r="A44" s="13" t="s">
+      <c r="H43" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I43" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="44" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A44" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B44" s="13" t="s">
+      <c r="B44" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C44" s="14">
-        <v>1</v>
-      </c>
-      <c r="D44" s="14">
-        <v>1</v>
-      </c>
-      <c r="E44" s="15">
-        <v>14</v>
-      </c>
-      <c r="F44" s="16">
+      <c r="C44" s="20">
+        <v>1</v>
+      </c>
+      <c r="D44" s="20">
+        <v>1</v>
+      </c>
+      <c r="E44" s="21">
+        <v>14</v>
+      </c>
+      <c r="F44" s="22">
         <v>0.027</v>
       </c>
-      <c r="G44" s="14">
+      <c r="G44" s="20">
         <v>12</v>
       </c>
-      <c r="H44" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I44" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1" spans="1:9">
-      <c r="A45" s="13" t="s">
+      <c r="H44" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I44" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="45" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A45" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B45" s="13" t="s">
+      <c r="B45" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C45" s="14">
-        <v>1</v>
-      </c>
-      <c r="D45" s="14">
+      <c r="C45" s="20">
+        <v>1</v>
+      </c>
+      <c r="D45" s="20">
         <v>0</v>
       </c>
-      <c r="E45" s="15">
-        <v>8</v>
-      </c>
-      <c r="F45" s="16">
+      <c r="E45" s="21">
+        <v>8</v>
+      </c>
+      <c r="F45" s="22">
         <v>0.028</v>
       </c>
-      <c r="G45" s="14">
+      <c r="G45" s="20">
         <v>10</v>
       </c>
-      <c r="H45" s="17"/>
-      <c r="I45" s="18">
+      <c r="H45" s="23"/>
+      <c r="I45" s="24">
         <v>7200</v>
       </c>
     </row>
@@ -3122,88 +3150,88 @@
         <v>7200</v>
       </c>
     </row>
-    <row r="49" ht="22" customHeight="1" spans="1:9">
-      <c r="A49" s="13" t="s">
+    <row r="49" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A49" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B49" s="13" t="s">
+      <c r="B49" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="C49" s="14">
-        <v>1</v>
-      </c>
-      <c r="D49" s="14">
-        <v>1</v>
-      </c>
-      <c r="E49" s="15">
+      <c r="C49" s="20">
+        <v>1</v>
+      </c>
+      <c r="D49" s="20">
+        <v>1</v>
+      </c>
+      <c r="E49" s="21">
         <v>3</v>
       </c>
-      <c r="F49" s="16">
+      <c r="F49" s="22">
         <v>0.012</v>
       </c>
-      <c r="G49" s="14">
+      <c r="G49" s="20">
         <v>22</v>
       </c>
-      <c r="H49" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I49" s="18">
-        <v>7200</v>
-      </c>
-    </row>
-    <row r="50" ht="22" customHeight="1" spans="1:9">
-      <c r="A50" s="13" t="s">
+      <c r="H49" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I49" s="24">
+        <v>7200</v>
+      </c>
+    </row>
+    <row r="50" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A50" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B50" s="13" t="s">
+      <c r="B50" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="C50" s="14">
-        <v>1</v>
-      </c>
-      <c r="D50" s="14">
-        <v>1</v>
-      </c>
-      <c r="E50" s="15">
-        <v>14</v>
-      </c>
-      <c r="F50" s="16">
+      <c r="C50" s="20">
+        <v>1</v>
+      </c>
+      <c r="D50" s="20">
+        <v>1</v>
+      </c>
+      <c r="E50" s="21">
+        <v>14</v>
+      </c>
+      <c r="F50" s="22">
         <v>0.027</v>
       </c>
-      <c r="G50" s="14">
+      <c r="G50" s="20">
         <v>12</v>
       </c>
-      <c r="H50" s="17">
-        <v>3600</v>
-      </c>
-      <c r="I50" s="18">
-        <v>3600</v>
-      </c>
-    </row>
-    <row r="51" ht="22" customHeight="1" spans="1:9">
-      <c r="A51" s="13" t="s">
+      <c r="H50" s="23">
+        <v>3600</v>
+      </c>
+      <c r="I50" s="24">
+        <v>3600</v>
+      </c>
+    </row>
+    <row r="51" s="10" customFormat="1" ht="22" customHeight="1" spans="1:9">
+      <c r="A51" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B51" s="13" t="s">
+      <c r="B51" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C51" s="14">
-        <v>1</v>
-      </c>
-      <c r="D51" s="14">
+      <c r="C51" s="20">
+        <v>1</v>
+      </c>
+      <c r="D51" s="20">
         <v>0</v>
       </c>
-      <c r="E51" s="15">
-        <v>8</v>
-      </c>
-      <c r="F51" s="16">
+      <c r="E51" s="21">
+        <v>8</v>
+      </c>
+      <c r="F51" s="22">
         <v>0.028</v>
       </c>
-      <c r="G51" s="14">
+      <c r="G51" s="20">
         <v>10</v>
       </c>
-      <c r="H51" s="17"/>
-      <c r="I51" s="18">
+      <c r="H51" s="23"/>
+      <c r="I51" s="24">
         <v>7200</v>
       </c>
     </row>
@@ -3302,7 +3330,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:I81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>

</xml_diff>